<commit_message>
Fix HKP API floor parsing bug (prefer tx.floor over floor_level.name) and sync all 3000 global transactions: 2026-08-03 12:04:11
</commit_message>
<xml_diff>
--- a/files/九龙-油麻地-原舍.xlsx
+++ b/files/九龙-油麻地-原舍.xlsx
@@ -266,10 +266,10 @@
     <xf numFmtId="0" fontId="16" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="17" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -6507,52 +6507,52 @@
     <row r="5" ht="58" customHeight="1">
       <c r="A5" s="19" t="inlineStr">
         <is>
-          <t>27&amp;28</t>
-        </is>
-      </c>
-      <c r="B5" s="20" t="inlineStr">
-        <is>
-          <t>A | 674呎 (2房)
+          <t>27</t>
+        </is>
+      </c>
+      <c r="B5" s="20" t="inlineStr"/>
+      <c r="C5" s="21" t="inlineStr">
+        <is>
+          <t>B | 286呎 (1房)
 -
 -
 (待售)</t>
         </is>
       </c>
-      <c r="C5" s="21" t="inlineStr"/>
-      <c r="D5" s="20" t="inlineStr">
-        <is>
-          <t>C | 572呎 (2房)
+      <c r="D5" s="20" t="inlineStr"/>
+      <c r="E5" s="21" t="inlineStr">
+        <is>
+          <t>D | 217呎 (开放式)
 -
 -
 (待售)</t>
         </is>
       </c>
-      <c r="E5" s="21" t="inlineStr"/>
     </row>
     <row r="6" ht="58" customHeight="1">
       <c r="A6" s="19" t="inlineStr">
         <is>
-          <t>27</t>
-        </is>
-      </c>
-      <c r="B6" s="21" t="inlineStr"/>
-      <c r="C6" s="20" t="inlineStr">
-        <is>
-          <t>B | 286呎 (1房)
+          <t>27&amp;28</t>
+        </is>
+      </c>
+      <c r="B6" s="21" t="inlineStr">
+        <is>
+          <t>A | 674呎 (2房)
 -
 -
 (待售)</t>
         </is>
       </c>
-      <c r="D6" s="21" t="inlineStr"/>
-      <c r="E6" s="20" t="inlineStr">
-        <is>
-          <t>D | 217呎 (开放式)
+      <c r="C6" s="20" t="inlineStr"/>
+      <c r="D6" s="21" t="inlineStr">
+        <is>
+          <t>C | 572呎 (2房)
 -
 -
 (待售)</t>
         </is>
       </c>
+      <c r="E6" s="20" t="inlineStr"/>
     </row>
     <row r="7" ht="58" customHeight="1">
       <c r="A7" s="19" t="inlineStr">
@@ -6560,7 +6560,7 @@
           <t>26</t>
         </is>
       </c>
-      <c r="B7" s="20" t="inlineStr">
+      <c r="B7" s="21" t="inlineStr">
         <is>
           <t>A | 304呎 (1房)
 -
@@ -6568,7 +6568,7 @@
 (待售)</t>
         </is>
       </c>
-      <c r="C7" s="20" t="inlineStr">
+      <c r="C7" s="21" t="inlineStr">
         <is>
           <t>B | 286呎 (1房)
 -
@@ -6576,7 +6576,7 @@
 (待售)</t>
         </is>
       </c>
-      <c r="D7" s="20" t="inlineStr">
+      <c r="D7" s="21" t="inlineStr">
         <is>
           <t>C | 318呎 (1房)
 -
@@ -6584,7 +6584,7 @@
 (待售)</t>
         </is>
       </c>
-      <c r="E7" s="20" t="inlineStr">
+      <c r="E7" s="21" t="inlineStr">
         <is>
           <t>D | 218呎 (开放式)
 -
@@ -6599,7 +6599,7 @@
           <t>25</t>
         </is>
       </c>
-      <c r="B8" s="20" t="inlineStr">
+      <c r="B8" s="21" t="inlineStr">
         <is>
           <t>A | 304呎 (1房)
 -
@@ -6607,7 +6607,7 @@
 (待售)</t>
         </is>
       </c>
-      <c r="C8" s="20" t="inlineStr">
+      <c r="C8" s="21" t="inlineStr">
         <is>
           <t>B | 286呎 (1房)
 -
@@ -6615,7 +6615,7 @@
 (待售)</t>
         </is>
       </c>
-      <c r="D8" s="20" t="inlineStr">
+      <c r="D8" s="21" t="inlineStr">
         <is>
           <t>C | 318呎 (1房)
 -
@@ -6623,7 +6623,7 @@
 (待售)</t>
         </is>
       </c>
-      <c r="E8" s="20" t="inlineStr">
+      <c r="E8" s="21" t="inlineStr">
         <is>
           <t>D | 218呎 (开放式)
 -
@@ -6638,7 +6638,7 @@
           <t>23</t>
         </is>
       </c>
-      <c r="B9" s="20" t="inlineStr">
+      <c r="B9" s="21" t="inlineStr">
         <is>
           <t>A | 304呎 (1房)
 -
@@ -6646,7 +6646,7 @@
 (待售)</t>
         </is>
       </c>
-      <c r="C9" s="20" t="inlineStr">
+      <c r="C9" s="21" t="inlineStr">
         <is>
           <t>B | 286呎 (1房)
 -
@@ -6654,7 +6654,7 @@
 (待售)</t>
         </is>
       </c>
-      <c r="D9" s="20" t="inlineStr">
+      <c r="D9" s="21" t="inlineStr">
         <is>
           <t>C | 318呎 (1房)
 -
@@ -6662,7 +6662,7 @@
 (待售)</t>
         </is>
       </c>
-      <c r="E9" s="20" t="inlineStr">
+      <c r="E9" s="21" t="inlineStr">
         <is>
           <t>D | 218呎 (开放式)
 -
@@ -6677,7 +6677,7 @@
           <t>22</t>
         </is>
       </c>
-      <c r="B10" s="20" t="inlineStr">
+      <c r="B10" s="21" t="inlineStr">
         <is>
           <t>A | 304呎 (1房)
 -
@@ -6685,7 +6685,7 @@
 (待售)</t>
         </is>
       </c>
-      <c r="C10" s="20" t="inlineStr">
+      <c r="C10" s="21" t="inlineStr">
         <is>
           <t>B | 286呎 (1房)
 -
@@ -6693,7 +6693,7 @@
 (待售)</t>
         </is>
       </c>
-      <c r="D10" s="20" t="inlineStr">
+      <c r="D10" s="21" t="inlineStr">
         <is>
           <t>C | 318呎 (1房)
 -
@@ -6701,7 +6701,7 @@
 (待售)</t>
         </is>
       </c>
-      <c r="E10" s="20" t="inlineStr">
+      <c r="E10" s="21" t="inlineStr">
         <is>
           <t>D | 218呎 (开放式)
 -
@@ -6716,7 +6716,7 @@
           <t>21</t>
         </is>
       </c>
-      <c r="B11" s="20" t="inlineStr">
+      <c r="B11" s="21" t="inlineStr">
         <is>
           <t>A | 304呎 (1房)
 -
@@ -6724,7 +6724,7 @@
 (待售)</t>
         </is>
       </c>
-      <c r="C11" s="20" t="inlineStr">
+      <c r="C11" s="21" t="inlineStr">
         <is>
           <t>B | 286呎 (1房)
 -
@@ -6732,7 +6732,7 @@
 (待售)</t>
         </is>
       </c>
-      <c r="D11" s="20" t="inlineStr">
+      <c r="D11" s="21" t="inlineStr">
         <is>
           <t>C | 318呎 (1房)
 -
@@ -6740,7 +6740,7 @@
 (待售)</t>
         </is>
       </c>
-      <c r="E11" s="20" t="inlineStr">
+      <c r="E11" s="21" t="inlineStr">
         <is>
           <t>D | 218呎 (开放式)
 -
@@ -6755,7 +6755,7 @@
           <t>20</t>
         </is>
       </c>
-      <c r="B12" s="20" t="inlineStr">
+      <c r="B12" s="21" t="inlineStr">
         <is>
           <t>A | 304呎 (1房)
 -
@@ -6763,7 +6763,7 @@
 (待售)</t>
         </is>
       </c>
-      <c r="C12" s="20" t="inlineStr">
+      <c r="C12" s="21" t="inlineStr">
         <is>
           <t>B | 286呎 (1房)
 -
@@ -6771,7 +6771,7 @@
 (待售)</t>
         </is>
       </c>
-      <c r="D12" s="20" t="inlineStr">
+      <c r="D12" s="21" t="inlineStr">
         <is>
           <t>C | 318呎 (1房)
 -
@@ -6779,7 +6779,7 @@
 (待售)</t>
         </is>
       </c>
-      <c r="E12" s="20" t="inlineStr">
+      <c r="E12" s="21" t="inlineStr">
         <is>
           <t>D | 218呎 (开放式)
 -
@@ -6794,7 +6794,7 @@
           <t>19</t>
         </is>
       </c>
-      <c r="B13" s="20" t="inlineStr">
+      <c r="B13" s="21" t="inlineStr">
         <is>
           <t>A | 304呎 (1房)
 -
@@ -6802,7 +6802,7 @@
 (待售)</t>
         </is>
       </c>
-      <c r="C13" s="20" t="inlineStr">
+      <c r="C13" s="21" t="inlineStr">
         <is>
           <t>B | 286呎 (1房)
 -
@@ -6810,7 +6810,7 @@
 (待售)</t>
         </is>
       </c>
-      <c r="D13" s="20" t="inlineStr">
+      <c r="D13" s="21" t="inlineStr">
         <is>
           <t>C | 318呎 (1房)
 -
@@ -6818,7 +6818,7 @@
 (待售)</t>
         </is>
       </c>
-      <c r="E13" s="20" t="inlineStr">
+      <c r="E13" s="21" t="inlineStr">
         <is>
           <t>D | 218呎 (开放式)
 -
@@ -6833,7 +6833,7 @@
           <t>18</t>
         </is>
       </c>
-      <c r="B14" s="20" t="inlineStr">
+      <c r="B14" s="21" t="inlineStr">
         <is>
           <t>A | 304呎 (1房)
 -
@@ -6849,7 +6849,7 @@
 (在售)</t>
         </is>
       </c>
-      <c r="D14" s="20" t="inlineStr">
+      <c r="D14" s="21" t="inlineStr">
         <is>
           <t>C | 318呎 (1房)
 -
@@ -6857,7 +6857,7 @@
 (待售)</t>
         </is>
       </c>
-      <c r="E14" s="20" t="inlineStr">
+      <c r="E14" s="21" t="inlineStr">
         <is>
           <t>D | 218呎 (开放式)
 -
@@ -6872,7 +6872,7 @@
           <t>17</t>
         </is>
       </c>
-      <c r="B15" s="20" t="inlineStr">
+      <c r="B15" s="21" t="inlineStr">
         <is>
           <t>A | 304呎 (1房)
 -
@@ -6888,7 +6888,7 @@
 (在售)</t>
         </is>
       </c>
-      <c r="D15" s="20" t="inlineStr">
+      <c r="D15" s="21" t="inlineStr">
         <is>
           <t>C | 318呎 (1房)
 -
@@ -6896,7 +6896,7 @@
 (待售)</t>
         </is>
       </c>
-      <c r="E15" s="20" t="inlineStr">
+      <c r="E15" s="21" t="inlineStr">
         <is>
           <t>D | 218呎 (开放式)
 -
@@ -6958,7 +6958,7 @@
 (26年-07月-28日)</t>
         </is>
       </c>
-      <c r="C17" s="20" t="inlineStr">
+      <c r="C17" s="21" t="inlineStr">
         <is>
           <t>B | 286呎 (1房)
 -
@@ -6966,7 +6966,7 @@
 (待售)</t>
         </is>
       </c>
-      <c r="D17" s="20" t="inlineStr">
+      <c r="D17" s="21" t="inlineStr">
         <is>
           <t>C | 318呎 (1房)
 -
@@ -6974,7 +6974,7 @@
 (待售)</t>
         </is>
       </c>
-      <c r="E17" s="20" t="inlineStr">
+      <c r="E17" s="21" t="inlineStr">
         <is>
           <t>D | 218呎 (开放式)
 -
@@ -7075,7 +7075,7 @@
 (26年-07月-24日)</t>
         </is>
       </c>
-      <c r="C20" s="20" t="inlineStr">
+      <c r="C20" s="21" t="inlineStr">
         <is>
           <t>B | 286呎 (1房)
 -
@@ -7114,7 +7114,7 @@
 (26年-07月-16日)</t>
         </is>
       </c>
-      <c r="C21" s="20" t="inlineStr">
+      <c r="C21" s="21" t="inlineStr">
         <is>
           <t>B | 286呎 (1房)
 -
@@ -7153,7 +7153,7 @@
 (在售)</t>
         </is>
       </c>
-      <c r="C22" s="20" t="inlineStr">
+      <c r="C22" s="21" t="inlineStr">
         <is>
           <t>B | 286呎 (1房)
 -
@@ -7231,7 +7231,7 @@
 (在售)</t>
         </is>
       </c>
-      <c r="C24" s="20" t="inlineStr">
+      <c r="C24" s="21" t="inlineStr">
         <is>
           <t>B | 286呎 (1房)
 -
@@ -7239,7 +7239,7 @@
 (待售)</t>
         </is>
       </c>
-      <c r="D24" s="20" t="inlineStr">
+      <c r="D24" s="21" t="inlineStr">
         <is>
           <t>C | 318呎 (1房)
 -
@@ -7262,7 +7262,7 @@
           <t>5</t>
         </is>
       </c>
-      <c r="B25" s="20" t="inlineStr">
+      <c r="B25" s="21" t="inlineStr">
         <is>
           <t>A | 304呎 (1房)
 -
@@ -7270,7 +7270,7 @@
 (待售)</t>
         </is>
       </c>
-      <c r="C25" s="20" t="inlineStr">
+      <c r="C25" s="21" t="inlineStr">
         <is>
           <t>B | 286呎 (1房)
 -
@@ -7278,7 +7278,7 @@
 (待售)</t>
         </is>
       </c>
-      <c r="D25" s="20" t="inlineStr">
+      <c r="D25" s="21" t="inlineStr">
         <is>
           <t>C | 318呎 (1房)
 -
@@ -7286,7 +7286,7 @@
 (待售)</t>
         </is>
       </c>
-      <c r="E25" s="20" t="inlineStr">
+      <c r="E25" s="21" t="inlineStr">
         <is>
           <t>D | 218呎 (开放式)
 -
@@ -7301,7 +7301,7 @@
           <t>3</t>
         </is>
       </c>
-      <c r="B26" s="20" t="inlineStr">
+      <c r="B26" s="21" t="inlineStr">
         <is>
           <t>A | 267呎 (1房)
 -
@@ -7309,7 +7309,7 @@
 (待售)</t>
         </is>
       </c>
-      <c r="C26" s="20" t="inlineStr">
+      <c r="C26" s="21" t="inlineStr">
         <is>
           <t>B | 248呎 (1房)
 -
@@ -7317,7 +7317,7 @@
 (待售)</t>
         </is>
       </c>
-      <c r="D26" s="20" t="inlineStr">
+      <c r="D26" s="21" t="inlineStr">
         <is>
           <t>C | 280呎 (1房)
 -
@@ -7325,7 +7325,7 @@
 (待售)</t>
         </is>
       </c>
-      <c r="E26" s="20" t="inlineStr">
+      <c r="E26" s="21" t="inlineStr">
         <is>
           <t>D | 180呎 (开放式)
 -

</xml_diff>